<commit_message>
fix: rebuild final data from raw subagent output to fix task/acceptance mismatch
</commit_message>
<xml_diff>
--- a/kol-questions/examples/agent测试题50条示例.xlsx
+++ b/kol-questions/examples/agent测试题50条示例.xlsx
@@ -514,7 +514,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>做一个「链接转 Markdown 阅读器」（x2markdown）：粘贴 X 帖子 / YouTube 视频 / GitHub 仓库 / ArXiv 论文 / HuggingFace 模型的链接，一键采集原文或字幕并转为 Markdown 格式，附带排版优化。</t>
+          <t>为游戏《ToME4》实现一个自主游玩Agent。要求该Agent能通过游戏屏幕截图或内嵌API感知状态，输出键盘鼠标操作，在遇到BOSS时能自主评估敌我实力差距；当评估为劣势时，主动采取“逃跑到安全距离再回头攻击”的战术，直至击杀BOSS。最终需提交可运行的Agent代码、运行日志和击杀BOSS的录像。</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -557,7 +557,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>做一个「人生顾问」/「六边形战士」型 AI 助手 skill：在迷茫或遇到工作/生活难题时，它不会直接给答案，而是从多个维度（成长、情绪、决策、复盘等）引导提问与给建议，可作为持续可复用的 personal assistant skill。</t>
+          <t>编写一个Python脚本，通过蓝牙BLE连接一个廉价的智能戒指（如华强北常见的智能戒指），读取其加速度计/触摸数据，识别2种以上手势（如晃动、双击），并将手势映射为Vibe Coding常用快捷键（如Ctrl+Enter运行代码、Ctrl+S保存），模拟键盘事件发送到当前焦点窗口。要求使用Vibe Coding风格——先快速实现核心循环，再根据实际测试结果迭代修正手势识别阈值和映射逻辑。</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -600,7 +600,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>做一个完整可部署的网页/应用：先用 Plan 模式让多个 Agent 各自输出开发计划，再选最佳方案由 Agent 执行从设计到上线的全流程。</t>
+          <t>编写一个Python脚本，模拟两个AI agent（A和B）的循环协作与接管：A负责初始化B、运行一个简单测试（如计算两个数之和），并实现两个接入插件（如读取文件和写入日志）；然后B读取A的配置文件，将A的记忆（关键状态）保存为JSON文件，并终止A（结束A的当前循环）。之后从保存的记忆中恢复A，让A再次初始化B的升级版（B的版本号+1），循环共3轮。脚本需在每轮打印清晰的日志，包括A创建B、测试结果、B保存记忆并终止A、A恢复记忆并创建B的新版本等步骤。</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -643,7 +643,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>为公司/部门搭建一个「商品或服务上架图 / 报表」自动化 Agent：输入原始数据或图，自动完成处理流程（如抠图加签、数据清洗汇总、生成报表）并输出成品，替代原本需要手动抠图/手动整理的工作。</t>
+          <t>为一个屏幕尺寸为 1024x768 的老旧平板设备（模拟 iPad 2 的浏览器环境）开发一个在线时钟网页应用，要求：1) 页面能在老旧浏览器（如 Safari 5）上正常显示并每秒更新当前时间；2) 提供“夜间模式”开关，使用 localStorage 记住用户选择；3) 全程使用 AI 辅助编程（例如通过对话让 AI 生成代码），并至少迭代 3 个版本，每次迭代根据自测发现的问题进行修复。最终将代码和迭代记录（每次修改内容）提交到指定仓库。</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -681,7 +681,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>做一个「AI 虚拟家长/陪写作业」助手：孩子做作业时，AI 以家长口吻陪伴、答疑、检查作业并给予反馈，而不是直接替写答案，做成可运行的应用。</t>
+          <t>为知乎设计并实现一个 Chrome 扩展（Manifest V3，Vanilla JS），能够将知乎文章、回答、想法（pin）等至少三种内容类型导出为 Markdown 文件。要求：1）为每种内容类型独立编写 parser，通过 URL 路由分发；2）处理知乎的特殊 DOM 节点（链接卡片、图片懒加载占位符、视频嵌入等），导出后公式、代码块、链接卡片不丢失；3）解决长内容导出不全的问题（需自行定位真实原因，例如抓取接口或解析路径）。最终导出文件应能在 Obsidian 中正常显示。</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -719,7 +719,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>编写一个体积极小的 Windows 桌面小工具：可锁定/解锁指定软件窗口（阻止点击/拖动或定时锁屏），单文件绿色运行</t>
+          <t>方法，实现一个“语音输入小键盘”的可运行 Web 原型。要求：在网页中模拟一个三键小键盘：1号键为“按住说话”语音输入，按下时开始用麦克风录音/识别，松开后自动把识别出的中文文本插入当前输入框；2号键为“自定义短语”键，点击后插入预设短语；3号键为“快捷键触发”键，点击后触发一次页面内预置的快捷操作（例如清空输入框或切换输入模式）。开发过程中必须使用 Vibe Coding 方式：通过与 AI 编程助手对话生成代码，并记录完整的 prompt 过程。最终交付物包括可运行代码、使用说明和 prompt 记录文档。</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -762,7 +762,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>开发一个对账自动化小工具：导入银行账单和内部账目（Excel/CSV），自动比对金额/日期/流水找出差异并出对账结果</t>
+          <t>请用你擅长的任一技术栈（如 Python + Streamlit / Gradio / HTML 静态页等）构建一个「AI 数学学习工作台」原型：① 提供一个输入界面，允许用户录入课程/论文/项目/截止日期/当前卡住的知识点；② 内置一个可复用的「思维法」库，至少包含 10 个来自解题/效率/时间管理领域的策略（如‘拆解成子问题’‘类比已知模型’‘倒推法’‘番茄钟’等）；③ 当用户输入一个卡住的知识点时，系统能自动匹配最相关的 3 条思维法，并生成一条可执行的下一步行动建议；④ 全部数据可保存在本地文件（如 JSON），刷新后不丢失。请实际运行并展示界面截图或交互演示。</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -805,7 +805,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>开发一个 Chrome 扩展：识别网页中的日语片假名外来语词汇，为其标注罗马音/发音/对应来源语言以辅助阅读</t>
+          <t>实现一个“AI Coding Plan 比价网站”：页面需收录至少 19 家产品、85 个套餐，覆盖 Claude Code、Codex、Cursor、Copilot、TRAE、Qwen、OpenRouter 等；每个套餐展示价格、额度、刷新周期、Agent 能力、实际用量对比；AI 视频套餐需单独用 credits 维度计算并展示；网站需包含每日更新数据的功能（可通过定时脚本或手动录入后自动生成更新时间），并提供按产品/价格/额度/刷新周期筛选或排序的交互。</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -848,7 +848,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>构建家庭网络的数字孪生可视化：绘制网络拓扑，实时展示各设备在线/流量/延迟等状态</t>
+          <t>基于开源硬件（如 Arduino/ESP32）和 AI 工具，编写一份完整的《用 AI 给手机造一个身体》教程文档。文档需包含：材料清单、硬件组装步骤、电路接线图、手机控制程序（含代码）、AI 集成方法（如语音指令或自动决策），并让手机通过该外设实现“自主移动”功能。</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -890,7 +890,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>搭建一条自动化工作流：例如定时抓取指定信息→处理后写入表格/发到邮箱（可用 n8n/Dify/Zapier 或 coding agent）</t>
+          <t>请用 vibecoding 方式（借助 AI 辅助设计）完成一个“会打人的猫”久坐提醒神器的可制造方案，并生成全部设计文件。具体交付：1）OpenSCAD 脚本（含猫形外壳、可动拍打臂与安装孔，能渲染出装配图）；2）Arduino/ESP32 固件代码（使用 PIR 人体传感器检测久坐，通过舵机驱动猫爪拍打用户，并带蜂鸣器提醒，代码须逻辑完整、可编译）；3）电路接线图（SVG 格式，标注引脚连接）；4）物料清单（含型号、数量、大致价格）；5）README（含组装步骤和参数调优说明）。</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -932,7 +932,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>从零开发一个可玩的格斗小游戏，包含角色立绘、攻击/闪避动画、血条、胜负判定。</t>
+          <t>/ AI 对话式编程，从零做一个可玩的格斗小游戏（含角色立绘、攻击/闪避动画、血条、胜负判定），全程无需手写大量代码，用自然语言驱动 AI 完成。</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -1016,7 +1016,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>做一个「照片时间机器」应用：上传一张照片，AI 识别画面中的建筑/街道/人物主体与空间结构，分别生成该场景</t>
+          <t>做一个「照片时间机器」应用：上传一张照片，AI 识别画面中的建筑/街道/人物主体与空间结构，分别生成该场景几十年前（过去）和几年后（未来）的样子，而非简单套复古/未来滤镜。</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1226,7 +1226,7 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>开发一个完整可部署的网页/应用：先用 Plan 模式让多个 Agent 各自输出开发计划，再选最佳方案由 Agent 执行从设计到上线的全流程。</t>
+          <t>做一个完整可部署的网页/应用：先用 Plan 模式让多个 Agent 各自输出开发计划，再选最佳方案由 Agent 执行从设计到上线的全流程。</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
@@ -1268,7 +1268,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>搭建一个「商品或服务上架图 / 报表」自动化 Agent：输入原始数据或图，自动完成处理流程（如抠图加签、数据清洗汇总、生成报表）并输出成品，替代原本需要手动抠图/手动整理的工作。</t>
+          <t>为公司/部门搭建一个「商品或服务上架图 / 报表」自动化 Agent：输入原始数据或图，自动完成处理流程（如抠图加签、数据清洗汇总、生成报表）并输出成品，替代原本需要手动抠图/手动整理的工作。</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -1352,7 +1352,7 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>为自家开发一个图文并茂的「家族史」生成工具，要求从家族口述/照片素材自动整理时间线、生成章节与插图，并输出为可分享的电子书（PDF/网页）。</t>
+          <t>为自家制作一本图文并茂的「家族史」，要求从家族口述/照片素材自动整理时间线、生成章节与插图，并输出为可分享的电子书（PDF/网页）。</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -1394,7 +1394,7 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>开发一个「AI 陪伴」App，可开源运行，包含对话与长期记忆，并提交到 GitHub 仓库。</t>
+          <t>把「AI 陪伴」做成一个可开源运行的 App（含对话与长期记忆），并提交到 GitHub 仓库。</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
@@ -1478,7 +1478,7 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>开发一款可在微信/网页运行的小程序，功能为「个人生活记录」，并提供可运行版本。</t>
+          <t>从0开发一款可在微信/网页运行的小程序，功能为「个人生活记录」，并提供可运行版本。</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
@@ -1520,7 +1520,7 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>开发一个可本地部署的「AI 赛博女友」聊天应用，要求免费、无需付费 API Key。</t>
+          <t>做一个可本地部署的「AI 赛博女友」聊天应用，要求免费、无需付费 API Key。</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -1562,7 +1562,7 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>快速开发一个小型 G 站/网页产品，并在一周内获得第一批真实用户。</t>
+          <t>快速开发一个小型 G 站/网页产品（类似用 Kimi K3 做产品），并在一周内获得第一批真实用户。</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
@@ -1646,7 +1646,7 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>实现一个「给网页加可视化微调器」的功能：通过一句描述让网页动态增加可实时调节样式参数的界面，例如给目标网页注入一个可拖拽调节的样式控制面板。</t>
+          <t>（如 Codex）实现一个「给网页加可视化微调器」的功能：通过一句描述让网页动态增加可实时调节样式参数的界面。</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
@@ -1772,7 +1772,7 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>搭建一个个人网站（含首页、关于页、联系页，附带响应式布局和导航菜单），并部署上线。</t>
+          <t>（如 Claude/Cursor）从零搭建一个个人网站（含首页、关于页、联系页，附带响应式布局和导航菜单），并部署上线</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
@@ -1814,7 +1814,7 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>搭建一条自动搜集信息并定时推送的任务管线：例如定时抓取指定关键词的资讯/数据，自动去重整理后推送到指定渠道（邮件/IM/表格）。</t>
+          <t>用一个全自动化的 AI Agent（如 n8n + LLM 工作流）搭一条自动搜集信息并定时推送的任务管线</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
@@ -1940,7 +1940,7 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>给自己做一个可用的 App（或小程序），实现一个具体功能（如记账、打卡、待办清单）。</t>
+          <t>工具给自己做一个可用的 App（或小程序），实现一个具体功能（如记账、打卡、待办清单）</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -2108,7 +2108,7 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>完成一个真实的小项目（如自动整理文件、自动爬取整理某类信息、自动生成周报），作为完整可交付用例。</t>
+          <t>Agent 完成一个真实的小项目（如自动整理文件、自动爬取整理某类信息、自动生成周报），作为完整可交付用例</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
@@ -2150,7 +2150,7 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>开发一个能在一天内完成并运行的小项目（工具/小游戏/网站），并尽量让代码可读可维护。</t>
+          <t>在一天内完成一个能运行的小项目（工具/小游戏/网站），并尽量让代码可读可维护</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -2192,7 +2192,7 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>构建一个可运行的背单词 APP，实现单词库管理、测词/复习、学习进度记录，并能打包成可安装应用（模拟上架 5 个应用市场）。</t>
+          <t>构建一个可运行的背单词 APP：实现单词库管理、测词/复习、学习进度记录，并能打包成可安装应用（模拟上架 5 个应用市场）</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
@@ -2234,7 +2234,7 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>开发一个纯前端英语单词过关网页：显示单词→用户作答中文释义→正确过关进入下一题，含计分与进度。</t>
+          <t>生成一个纯前端英语单词过关网页：显示单词→用户作答中文释义→正确过关进入下一题，含计分与进度</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
@@ -2276,7 +2276,7 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>构建一个单机国际象棋游戏：实现完整棋规（走子、吃子、王车易位、升变、将杀判断），支持与 AI 人机对弈或本地双人，含悔棋/重开。</t>
+          <t>构建一个单机国际象棋游戏：实现完整棋规（走子、吃子、王车易位、升变、将杀判断），支持与 AI 人机对弈或本地双人，含悔棋/重开</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
@@ -2360,7 +2360,7 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>开发一个儿童数学出题器：可设置题数与难度，自动生成题目并判分，网页或可打印</t>
+          <t>快速生成一个儿童数学出题器：可设置题数与难度，自动生成题目并判分，网页或可打印</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
@@ -2444,7 +2444,7 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>开发一个对账自动化小工具：导入银行账单和内部账目（Excel/CSV），自动比对金额/日期/流水找出差异并出对账结果。</t>
+          <t>开发一个对账自动化小工具：导入银行账单和内部账目（Excel/CSV），自动比对金额/日期/流水找出差异并出对账结果</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
@@ -2486,7 +2486,7 @@
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>开发一个 Chrome 扩展：识别网页中的日语片假名外来语词汇，为其标注罗马音/发音/对应来源语言以辅助阅读。</t>
+          <t>开发一个 Chrome 扩展：识别网页中的日语片假名外来语词汇，为其标注罗马音/发音/对应来源语言以辅助阅读</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">

</xml_diff>